<commit_message>
Blood flows in the PFDA, PHxS and PFNA input spreadsheets revised for mass balance, including flow to lung tissue.
</commit_message>
<xml_diff>
--- a/Inputs/PFDA_template_parameters_Model.xlsx
+++ b/Inputs/PFDA_template_parameters_Model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24931"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/bernstein_amanda_epa_gov/Documents/Documents/PKWG_models/pbpk_template_project/Inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="78" documentId="13_ncr:1_{C63AA975-7954-4754-AC1D-939BBF5412ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C057820-2B86-42C8-9631-CB590D627930}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="13_ncr:1_{C63AA975-7954-4754-AC1D-939BBF5412ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80C0268E-B65A-4B2F-B67F-34160FF3418A}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="2595" yWindow="2460" windowWidth="25740" windowHeight="12795" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="FKimRecreateBW" sheetId="9" r:id="rId1"/>
@@ -797,14 +797,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -884,9 +882,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -924,7 +922,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1030,7 +1028,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1172,7 +1170,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1181,21 +1179,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ADCAA70-43B6-4F02-AE2A-67A6EACE5958}">
   <dimension ref="A1:G104"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.453125" customWidth="1"/>
-    <col min="3" max="3" width="26.81640625" customWidth="1"/>
-    <col min="4" max="4" width="13.08984375" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.42578125" customWidth="1"/>
+    <col min="3" max="3" width="26.85546875" customWidth="1"/>
+    <col min="4" max="4" width="13.140625" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1215,7 +1213,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1229,7 +1227,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1240,7 +1238,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1251,7 +1249,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -1268,7 +1266,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -1285,7 +1283,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -1299,7 +1297,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>20</v>
       </c>
@@ -1313,7 +1311,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>238</v>
       </c>
@@ -1330,7 +1328,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>135</v>
       </c>
@@ -1347,7 +1345,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>136</v>
       </c>
@@ -1364,7 +1362,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>173</v>
       </c>
@@ -1381,7 +1379,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>177</v>
       </c>
@@ -1398,7 +1396,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>165</v>
       </c>
@@ -1415,7 +1413,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>191</v>
       </c>
@@ -1427,13 +1425,13 @@
       </c>
       <c r="E15">
         <f>1-SUM(E76:E85)</f>
-        <v>-0.99224806201550408</v>
+        <v>0</v>
       </c>
       <c r="F15" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>194</v>
       </c>
@@ -1448,7 +1446,7 @@
         <v>0.70472000000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
@@ -1468,7 +1466,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>71</v>
       </c>
@@ -1488,7 +1486,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>27</v>
       </c>
@@ -1505,7 +1503,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
@@ -1519,7 +1517,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>230</v>
       </c>
@@ -1537,7 +1535,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>31</v>
       </c>
@@ -1551,7 +1549,7 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>33</v>
       </c>
@@ -1566,13 +1564,13 @@
       </c>
       <c r="E24">
         <f>F24/(G20^E20)</f>
-        <v>7297.3419818451703</v>
+        <v>14538.115421195416</v>
       </c>
       <c r="F24">
-        <v>2580</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+        <v>5140</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>43</v>
       </c>
@@ -1586,7 +1584,7 @@
         <v>0.65</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>141</v>
       </c>
@@ -1599,7 +1597,7 @@
       <c r="D26">
         <v>0</v>
       </c>
-      <c r="E26" s="4">
+      <c r="E26" s="3">
         <f>F26/(G20^E21)</f>
         <v>113844.19177103414</v>
       </c>
@@ -1607,7 +1605,7 @@
         <v>40250</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>142</v>
       </c>
@@ -1627,7 +1625,7 @@
         <v>30051</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>48</v>
       </c>
@@ -1651,7 +1649,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>143</v>
       </c>
@@ -1672,7 +1670,7 @@
         <v>0.68100000000000005</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>144</v>
       </c>
@@ -1686,7 +1684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>145</v>
       </c>
@@ -1707,7 +1705,7 @@
         <v>0.39100000000000001</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>52</v>
       </c>
@@ -1727,7 +1725,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>53</v>
       </c>
@@ -1741,7 +1739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>54</v>
       </c>
@@ -1755,7 +1753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>55</v>
       </c>
@@ -1769,7 +1767,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>166</v>
       </c>
@@ -1783,7 +1781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>57</v>
       </c>
@@ -1804,7 +1802,7 @@
         <v>0.75800000000000001</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>226</v>
       </c>
@@ -1818,7 +1816,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>227</v>
       </c>
@@ -1832,7 +1830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>228</v>
       </c>
@@ -1846,7 +1844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>146</v>
       </c>
@@ -1860,7 +1858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>147</v>
       </c>
@@ -1874,7 +1872,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>148</v>
       </c>
@@ -1888,7 +1886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>149</v>
       </c>
@@ -1902,7 +1900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>150</v>
       </c>
@@ -1916,7 +1914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>151</v>
       </c>
@@ -1930,7 +1928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>152</v>
       </c>
@@ -1944,7 +1942,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>153</v>
       </c>
@@ -1958,7 +1956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>38</v>
       </c>
@@ -1969,7 +1967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>169</v>
       </c>
@@ -1980,7 +1978,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>40</v>
       </c>
@@ -1991,7 +1989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>183</v>
       </c>
@@ -2006,13 +2004,13 @@
       </c>
       <c r="E52">
         <f>F52/F24</f>
-        <v>0.10077519379844961</v>
+        <v>5.0583657587548639E-2</v>
       </c>
       <c r="F52">
         <v>260</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>161</v>
       </c>
@@ -2026,7 +2024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>162</v>
       </c>
@@ -2037,7 +2035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>197</v>
       </c>
@@ -2051,7 +2049,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>199</v>
       </c>
@@ -2065,7 +2063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>233</v>
       </c>
@@ -2082,7 +2080,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>42</v>
       </c>
@@ -2096,7 +2094,7 @@
         <v>1.22E-4</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>0</v>
       </c>
@@ -2113,7 +2111,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>81</v>
       </c>
@@ -2134,7 +2132,7 @@
         <v>20.399999999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>137</v>
       </c>
@@ -2148,7 +2146,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>139</v>
       </c>
@@ -2162,7 +2160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>84</v>
       </c>
@@ -2176,7 +2174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>91</v>
       </c>
@@ -2197,7 +2195,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>92</v>
       </c>
@@ -2218,7 +2216,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>93</v>
       </c>
@@ -2239,7 +2237,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>94</v>
       </c>
@@ -2260,7 +2258,7 @@
         <v>0.18</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>95</v>
       </c>
@@ -2281,7 +2279,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>96</v>
       </c>
@@ -2302,7 +2300,7 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>97</v>
       </c>
@@ -2316,7 +2314,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>98</v>
       </c>
@@ -2330,7 +2328,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>99</v>
       </c>
@@ -2344,7 +2342,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>100</v>
       </c>
@@ -2358,7 +2356,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>154</v>
       </c>
@@ -2379,7 +2377,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>105</v>
       </c>
@@ -2394,13 +2392,13 @@
       </c>
       <c r="E76">
         <f>F76/F24</f>
-        <v>0.1744186046511628</v>
+        <v>8.7548638132295714E-2</v>
       </c>
       <c r="F76">
         <v>450</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>106</v>
       </c>
@@ -2415,13 +2413,13 @@
       </c>
       <c r="E77">
         <f>F77/F24</f>
-        <v>0.32093023255813952</v>
+        <v>0.16108949416342414</v>
       </c>
       <c r="F77">
         <v>828</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>107</v>
       </c>
@@ -2436,13 +2434,13 @@
       </c>
       <c r="E78">
         <f>F78/F24</f>
-        <v>0.20155038759689922</v>
+        <v>0.10116731517509728</v>
       </c>
       <c r="F78">
         <v>520</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>108</v>
       </c>
@@ -2455,15 +2453,15 @@
       <c r="D79">
         <v>0</v>
       </c>
-      <c r="E79" s="5">
+      <c r="E79" s="4">
         <f>F79/F24</f>
-        <v>1</v>
+        <v>0.50194552529182879</v>
       </c>
       <c r="F79">
         <v>2580</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>109</v>
       </c>
@@ -2478,13 +2476,13 @@
       </c>
       <c r="E80">
         <f>F80/F24</f>
-        <v>9.0697674418604657E-2</v>
+        <v>4.5525291828793772E-2</v>
       </c>
       <c r="F80">
         <v>234</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>110</v>
       </c>
@@ -2498,7 +2496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>111</v>
       </c>
@@ -2512,7 +2510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>112</v>
       </c>
@@ -2526,7 +2524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>113</v>
       </c>
@@ -2540,7 +2538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>156</v>
       </c>
@@ -2553,15 +2551,15 @@
       <c r="D85">
         <v>0</v>
       </c>
-      <c r="E85" s="6">
+      <c r="E85">
         <f>F85/F24</f>
-        <v>0.20465116279069767</v>
+        <v>0.10272373540856031</v>
       </c>
       <c r="F85">
         <v>528</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>122</v>
       </c>
@@ -2571,9 +2569,8 @@
       <c r="D86">
         <v>1</v>
       </c>
-      <c r="E86" s="6"/>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.35">
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>123</v>
       </c>
@@ -2587,7 +2584,7 @@
         <v>1.0200000000000001E-2</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>124</v>
       </c>
@@ -2601,7 +2598,7 @@
         <v>0.60699999999999998</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>125</v>
       </c>
@@ -2615,7 +2612,7 @@
         <v>0.23280000000000001</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>126</v>
       </c>
@@ -2629,7 +2626,7 @@
         <v>0.1002</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>127</v>
       </c>
@@ -2643,7 +2640,7 @@
         <v>4.36E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>128</v>
       </c>
@@ -2654,7 +2651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>129</v>
       </c>
@@ -2665,7 +2662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>130</v>
       </c>
@@ -2676,7 +2673,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>131</v>
       </c>
@@ -2687,7 +2684,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>158</v>
       </c>
@@ -2701,7 +2698,7 @@
         <v>2.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>0</v>
       </c>
@@ -2718,7 +2715,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>35</v>
       </c>
@@ -2726,7 +2723,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>0</v>
       </c>
@@ -2741,7 +2738,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>75</v>
       </c>
@@ -2749,7 +2746,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>77</v>
       </c>
@@ -2757,7 +2754,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>79</v>
       </c>
@@ -2796,10 +2793,59 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </e3f09c3df709400db2417a7161762d62>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3272,73 +3318,20 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </e3f09c3df709400db2417a7161762d62>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DC8FD00-95C1-4E09-89D4-FF0C8178E817}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -3348,14 +3341,38 @@
     <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
     <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DC8FD00-95C1-4E09-89D4-FF0C8178E817}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+    <ds:schemaRef ds:uri="41d9f072-86bf-4c63-b117-debf50ff4701"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>